<commit_message>
Weekly data update: training.xlsx
</commit_message>
<xml_diff>
--- a/training.xlsx
+++ b/training.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Shared drives\Synergy Safety Group\DEN\Dashboard\Weekly Dashboards\AN-Transport\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F54E244E-6907-407B-A17B-F9711AE049D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A77CE58F-4036-4348-9E23-1F439C3B592B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="1215" windowWidth="21930" windowHeight="14985" xr2:uid="{5CACA9A1-03A8-4E05-97D6-00ACC1325A4A}"/>
+    <workbookView xWindow="2730" yWindow="2730" windowWidth="43200" windowHeight="11235" xr2:uid="{5CACA9A1-03A8-4E05-97D6-00ACC1325A4A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21445,16 +21445,16 @@
         <v>30</v>
       </c>
       <c r="G675" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H675" s="2">
-        <v>0</v>
+        <v>6.8402777777777776E-3</v>
       </c>
       <c r="I675" s="1">
         <v>46176.506249999999</v>
       </c>
       <c r="J675">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K675" t="s">
         <v>11</v>
@@ -21547,7 +21547,7 @@
         <v>46176.507638888892</v>
       </c>
       <c r="J678">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K678" t="s">
         <v>11</v>
@@ -21602,16 +21602,16 @@
         <v>30</v>
       </c>
       <c r="G680" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H680">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="H680" s="2">
+        <v>1.3321759259259259E-2</v>
       </c>
       <c r="I680" s="1">
         <v>46176.508333333331</v>
       </c>
       <c r="J680">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K680" t="s">
         <v>11</v>
@@ -21643,7 +21643,7 @@
         <v>46176.509027777778</v>
       </c>
       <c r="J681">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K681" t="s">
         <v>11</v>
@@ -21716,7 +21716,7 @@
         <v>46176.509722222225</v>
       </c>
       <c r="J684">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K684" t="s">
         <v>11</v>
@@ -21748,7 +21748,7 @@
         <v>46176.510416666664</v>
       </c>
       <c r="J685">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K685" t="s">
         <v>11</v>
@@ -21844,7 +21844,7 @@
         <v>46176.511111111111</v>
       </c>
       <c r="J688">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K688" t="s">
         <v>11</v>
@@ -21876,7 +21876,7 @@
         <v>46176.511111111111</v>
       </c>
       <c r="J689">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K689" t="s">
         <v>11</v>
@@ -21940,16 +21940,16 @@
         <v>30</v>
       </c>
       <c r="G692" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H692" s="2">
-        <v>0</v>
+        <v>8.2060185185185187E-3</v>
       </c>
       <c r="I692" s="1">
         <v>46176.511805555558</v>
       </c>
       <c r="J692">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K692" t="s">
         <v>11</v>
@@ -22045,7 +22045,7 @@
         <v>46176.513194444444</v>
       </c>
       <c r="J695">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K695" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
Update training.xlsx (weekly dashboard refresh)
</commit_message>
<xml_diff>
--- a/training.xlsx
+++ b/training.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Shared drives\Synergy Safety Group\DEN\Dashboard\Weekly Dashboards\AN-Transport\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BBB42B85-2164-4C9F-B97A-73A3B0E7898B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{52FF328B-34E3-4AD9-B42D-E75B9121A19D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="15720" xr2:uid="{5CACA9A1-03A8-4E05-97D6-00ACC1325A4A}"/>
+    <workbookView xWindow="3585" yWindow="3585" windowWidth="43200" windowHeight="11235" xr2:uid="{5CACA9A1-03A8-4E05-97D6-00ACC1325A4A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -739,7 +739,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79F75797-B237-43B3-82D5-68EF721AABF0}">
-  <dimension ref="B1:K7400"/>
+  <dimension ref="A1:K7400"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
@@ -754,39 +754,39 @@
     <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>33</v>
       </c>
@@ -818,7 +818,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>33</v>
       </c>
@@ -850,7 +850,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>33</v>
       </c>
@@ -882,7 +882,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>33</v>
       </c>
@@ -914,7 +914,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="H6" s="2"/>
       <c r="I6" s="1"/>
       <c r="J6" s="2"/>
@@ -922,7 +922,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>33</v>
       </c>
@@ -954,7 +954,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>33</v>
       </c>
@@ -986,7 +986,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>33</v>
       </c>
@@ -1018,7 +1018,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>33</v>
       </c>
@@ -1050,7 +1050,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>33</v>
       </c>
@@ -1082,7 +1082,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>33</v>
       </c>
@@ -1114,7 +1114,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>33</v>
       </c>
@@ -1146,7 +1146,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>33</v>
       </c>
@@ -1178,7 +1178,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
         <v>33</v>
       </c>
@@ -1210,7 +1210,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>33</v>
       </c>
@@ -23599,10 +23599,10 @@
         <v>29</v>
       </c>
       <c r="G747" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H747" s="2">
-        <v>0</v>
+        <v>5.7407407407407407E-3</v>
       </c>
       <c r="I747" s="1">
         <v>46237.628125000003</v>
@@ -23791,10 +23791,10 @@
         <v>29</v>
       </c>
       <c r="G753" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H753" s="2">
-        <v>0</v>
+        <v>5.9722222222222225E-3</v>
       </c>
       <c r="I753" s="1">
         <v>46237.630208333336</v>
@@ -23823,10 +23823,10 @@
         <v>29</v>
       </c>
       <c r="G754" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H754" s="2">
-        <v>0</v>
+        <v>5.9837962962962961E-3</v>
       </c>
       <c r="I754" s="1">
         <v>46237.630902777775</v>
@@ -23887,10 +23887,10 @@
         <v>29</v>
       </c>
       <c r="G756" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H756" s="2">
-        <v>0</v>
+        <v>7.0486111111111114E-3</v>
       </c>
       <c r="I756" s="1">
         <v>46237.631597222222</v>
@@ -23951,10 +23951,10 @@
         <v>29</v>
       </c>
       <c r="G758" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H758" s="2">
-        <v>0</v>
+        <v>6.3310185185185188E-3</v>
       </c>
       <c r="I758" s="1">
         <v>46237.632986111108</v>
@@ -24015,10 +24015,10 @@
         <v>29</v>
       </c>
       <c r="G760" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H760" s="2">
-        <v>0</v>
+        <v>7.7546296296296295E-3</v>
       </c>
       <c r="I760" s="1">
         <v>46237.633680555555</v>
@@ -24443,6 +24443,7 @@
       <c r="K781" s="1"/>
     </row>
     <row r="782" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="H782" s="2"/>
       <c r="I782" s="1"/>
       <c r="J782" s="2"/>
       <c r="K782" s="1"/>
@@ -24982,6 +24983,7 @@
       <c r="K871" s="1"/>
     </row>
     <row r="872" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H872" s="2"/>
       <c r="I872" s="1"/>
       <c r="J872" s="2"/>
       <c r="K872" s="1"/>
@@ -25347,6 +25349,7 @@
       <c r="K932" s="1"/>
     </row>
     <row r="933" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H933" s="2"/>
       <c r="I933" s="1"/>
       <c r="J933" s="2"/>
       <c r="K933" s="1"/>
@@ -25592,6 +25595,7 @@
       <c r="K973" s="1"/>
     </row>
     <row r="974" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H974" s="2"/>
       <c r="I974" s="1"/>
       <c r="J974" s="2"/>
       <c r="K974" s="1"/>

</xml_diff>